<commit_message>
Release 0.3.0: giroconto cross-broker matching (Ris. 60/E)
- Matching automatico cross-broker in forex_gains.py: un wire-out abbinato a un wire-in positivo su un altro conto (stessa valuta, importo entro 0,01 USD, settle date entro ±3 giorni lavorativi) genera un evento TRANSFER che sposta i lotti USD dalla coda LIFO del conto di origine a quella di destinazione cronologicamente, preservando data di acquisizione e cambio BCE originali. Nessuna plusvalenza artificiale sulla data del giroconto (Ris. AdE 60/E del 09/12/2024).
- pyproject.toml: version bump 0.2.0 → 0.3.0.
- README: URL jsdelivr pinnate a @v0.3.0 (evita staleness 7gg cache @master); rimossa riga "Giroconto cross-broker in USD" da §Limitazioni note.
- CHANGELOG: sezione [0.3.0] — 2026-04-19.
- examples/: rigenerati via scripts/gen_examples.py. L'unico cambio di contenuto e' su mascetti/decaf_2025.yaml (scompare la plusvalenza artificiale di €1,78 del 10/25).
</commit_message>
<xml_diff>
--- a/examples/mascetti/decaf_2025.xlsx
+++ b/examples/mascetti/decaf_2025.xlsx
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>488.64</v>
+        <v>486.86</v>
       </c>
     </row>
     <row r="15">
@@ -1842,7 +1842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2189,72 +2189,23 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>EUR.USD</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Plusvalenza valutaria USD (LIFO per conto)</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2025-10-25</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>2400</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>2066.83</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>2065.05</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="J7" t="n">
-        <v>1.1612</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="4" t="n">
-        <v>0</v>
-      </c>
+      <c r="I7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="I8" s="6" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
         <is>
           <t>NETTO</t>
         </is>
       </c>
-      <c r="I9" s="4" t="n">
-        <v>488.64</v>
+      <c r="I8" s="4" t="n">
+        <v>486.86</v>
       </c>
     </row>
   </sheetData>
@@ -8977,10 +8928,10 @@
         </is>
       </c>
       <c r="B304" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C304" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D304" t="n">
         <v>1.0389</v>
@@ -8999,10 +8950,10 @@
         </is>
       </c>
       <c r="B305" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C305" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D305" t="n">
         <v>1.0389</v>
@@ -9021,10 +8972,10 @@
         </is>
       </c>
       <c r="B306" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C306" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D306" t="n">
         <v>1.0389</v>
@@ -9043,10 +8994,10 @@
         </is>
       </c>
       <c r="B307" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C307" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D307" t="n">
         <v>1.0389</v>
@@ -9065,10 +9016,10 @@
         </is>
       </c>
       <c r="B308" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C308" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D308" t="n">
         <v>1.0389</v>
@@ -9087,10 +9038,10 @@
         </is>
       </c>
       <c r="B309" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C309" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D309" t="n">
         <v>1.0389</v>
@@ -9105,10 +9056,10 @@
         </is>
       </c>
       <c r="B310" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C310" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D310" t="n">
         <v>1.0389</v>
@@ -9123,10 +9074,10 @@
         </is>
       </c>
       <c r="B311" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C311" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D311" t="n">
         <v>1.0389</v>
@@ -9145,10 +9096,10 @@
         </is>
       </c>
       <c r="B312" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C312" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D312" t="n">
         <v>1.0389</v>
@@ -9167,10 +9118,10 @@
         </is>
       </c>
       <c r="B313" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C313" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D313" t="n">
         <v>1.0389</v>
@@ -9189,10 +9140,10 @@
         </is>
       </c>
       <c r="B314" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C314" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D314" t="n">
         <v>1.0389</v>
@@ -9211,10 +9162,10 @@
         </is>
       </c>
       <c r="B315" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C315" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D315" t="n">
         <v>1.0389</v>
@@ -9233,10 +9184,10 @@
         </is>
       </c>
       <c r="B316" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C316" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D316" t="n">
         <v>1.0389</v>
@@ -9251,10 +9202,10 @@
         </is>
       </c>
       <c r="B317" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C317" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D317" t="n">
         <v>1.0389</v>
@@ -9269,10 +9220,10 @@
         </is>
       </c>
       <c r="B318" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C318" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D318" t="n">
         <v>1.0389</v>
@@ -9291,10 +9242,10 @@
         </is>
       </c>
       <c r="B319" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C319" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D319" t="n">
         <v>1.0389</v>
@@ -9313,10 +9264,10 @@
         </is>
       </c>
       <c r="B320" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C320" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D320" t="n">
         <v>1.0389</v>
@@ -9335,10 +9286,10 @@
         </is>
       </c>
       <c r="B321" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C321" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D321" t="n">
         <v>1.0389</v>
@@ -9357,10 +9308,10 @@
         </is>
       </c>
       <c r="B322" s="4" t="n">
-        <v>13708.5</v>
+        <v>16108.5</v>
       </c>
       <c r="C322" s="4" t="n">
-        <v>13195.20646838002</v>
+        <v>15505.3421888536</v>
       </c>
       <c r="D322" t="n">
         <v>1.0389</v>
@@ -9379,10 +9330,10 @@
         </is>
       </c>
       <c r="B323" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C323" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D323" t="n">
         <v>1.0389</v>
@@ -9397,10 +9348,10 @@
         </is>
       </c>
       <c r="B324" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C324" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D324" t="n">
         <v>1.0389</v>
@@ -9415,10 +9366,10 @@
         </is>
       </c>
       <c r="B325" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C325" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D325" t="n">
         <v>1.0389</v>
@@ -9437,10 +9388,10 @@
         </is>
       </c>
       <c r="B326" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C326" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D326" t="n">
         <v>1.0389</v>
@@ -9459,10 +9410,10 @@
         </is>
       </c>
       <c r="B327" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C327" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D327" t="n">
         <v>1.0389</v>
@@ -9481,10 +9432,10 @@
         </is>
       </c>
       <c r="B328" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C328" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D328" t="n">
         <v>1.0389</v>
@@ -9503,10 +9454,10 @@
         </is>
       </c>
       <c r="B329" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C329" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D329" t="n">
         <v>1.0389</v>
@@ -9525,10 +9476,10 @@
         </is>
       </c>
       <c r="B330" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C330" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D330" t="n">
         <v>1.0389</v>
@@ -9543,10 +9494,10 @@
         </is>
       </c>
       <c r="B331" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C331" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D331" t="n">
         <v>1.0389</v>
@@ -9561,10 +9512,10 @@
         </is>
       </c>
       <c r="B332" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C332" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D332" t="n">
         <v>1.0389</v>
@@ -9583,10 +9534,10 @@
         </is>
       </c>
       <c r="B333" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C333" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D333" t="n">
         <v>1.0389</v>
@@ -9605,10 +9556,10 @@
         </is>
       </c>
       <c r="B334" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C334" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D334" t="n">
         <v>1.0389</v>
@@ -9627,10 +9578,10 @@
         </is>
       </c>
       <c r="B335" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C335" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D335" t="n">
         <v>1.0389</v>
@@ -9649,10 +9600,10 @@
         </is>
       </c>
       <c r="B336" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C336" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D336" t="n">
         <v>1.0389</v>
@@ -9671,10 +9622,10 @@
         </is>
       </c>
       <c r="B337" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C337" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D337" t="n">
         <v>1.0389</v>
@@ -9689,10 +9640,10 @@
         </is>
       </c>
       <c r="B338" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C338" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D338" t="n">
         <v>1.0389</v>
@@ -9707,10 +9658,10 @@
         </is>
       </c>
       <c r="B339" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C339" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D339" t="n">
         <v>1.0389</v>
@@ -9729,10 +9680,10 @@
         </is>
       </c>
       <c r="B340" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C340" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D340" t="n">
         <v>1.0389</v>
@@ -9751,10 +9702,10 @@
         </is>
       </c>
       <c r="B341" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C341" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D341" t="n">
         <v>1.0389</v>
@@ -9773,10 +9724,10 @@
         </is>
       </c>
       <c r="B342" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C342" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D342" t="n">
         <v>1.0389</v>
@@ -9795,10 +9746,10 @@
         </is>
       </c>
       <c r="B343" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C343" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D343" t="n">
         <v>1.0389</v>
@@ -9817,10 +9768,10 @@
         </is>
       </c>
       <c r="B344" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C344" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D344" t="n">
         <v>1.0389</v>
@@ -9835,10 +9786,10 @@
         </is>
       </c>
       <c r="B345" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C345" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D345" t="n">
         <v>1.0389</v>
@@ -9853,10 +9804,10 @@
         </is>
       </c>
       <c r="B346" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C346" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D346" t="n">
         <v>1.0389</v>
@@ -9871,10 +9822,10 @@
         </is>
       </c>
       <c r="B347" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C347" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D347" t="n">
         <v>1.0389</v>
@@ -9893,10 +9844,10 @@
         </is>
       </c>
       <c r="B348" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C348" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D348" t="n">
         <v>1.0389</v>
@@ -9915,10 +9866,10 @@
         </is>
       </c>
       <c r="B349" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C349" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D349" t="n">
         <v>1.0389</v>
@@ -9937,10 +9888,10 @@
         </is>
       </c>
       <c r="B350" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C350" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D350" t="n">
         <v>1.0389</v>
@@ -9959,10 +9910,10 @@
         </is>
       </c>
       <c r="B351" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C351" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D351" t="n">
         <v>1.0389</v>
@@ -9977,10 +9928,10 @@
         </is>
       </c>
       <c r="B352" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C352" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D352" t="n">
         <v>1.0389</v>
@@ -9995,10 +9946,10 @@
         </is>
       </c>
       <c r="B353" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C353" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D353" t="n">
         <v>1.0389</v>
@@ -10017,10 +9968,10 @@
         </is>
       </c>
       <c r="B354" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C354" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D354" t="n">
         <v>1.0389</v>
@@ -10039,10 +9990,10 @@
         </is>
       </c>
       <c r="B355" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C355" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D355" t="n">
         <v>1.0389</v>
@@ -10061,10 +10012,10 @@
         </is>
       </c>
       <c r="B356" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C356" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D356" t="n">
         <v>1.0389</v>
@@ -10083,10 +10034,10 @@
         </is>
       </c>
       <c r="B357" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C357" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D357" t="n">
         <v>1.0389</v>
@@ -10105,10 +10056,10 @@
         </is>
       </c>
       <c r="B358" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C358" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D358" t="n">
         <v>1.0389</v>
@@ -10123,10 +10074,10 @@
         </is>
       </c>
       <c r="B359" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C359" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D359" t="n">
         <v>1.0389</v>
@@ -10141,10 +10092,10 @@
         </is>
       </c>
       <c r="B360" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C360" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D360" t="n">
         <v>1.0389</v>
@@ -10163,10 +10114,10 @@
         </is>
       </c>
       <c r="B361" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C361" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D361" t="n">
         <v>1.0389</v>
@@ -10185,10 +10136,10 @@
         </is>
       </c>
       <c r="B362" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C362" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D362" t="n">
         <v>1.0389</v>
@@ -10207,10 +10158,10 @@
         </is>
       </c>
       <c r="B363" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C363" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D363" t="n">
         <v>1.0389</v>
@@ -10225,10 +10176,10 @@
         </is>
       </c>
       <c r="B364" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C364" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D364" t="n">
         <v>1.0389</v>
@@ -10243,10 +10194,10 @@
         </is>
       </c>
       <c r="B365" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C365" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D365" t="n">
         <v>1.0389</v>
@@ -10261,10 +10212,10 @@
         </is>
       </c>
       <c r="B366" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C366" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D366" t="n">
         <v>1.0389</v>
@@ -10279,10 +10230,10 @@
         </is>
       </c>
       <c r="B367" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C367" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D367" t="n">
         <v>1.0389</v>
@@ -10301,10 +10252,10 @@
         </is>
       </c>
       <c r="B368" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C368" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D368" t="n">
         <v>1.0389</v>
@@ -10323,10 +10274,10 @@
         </is>
       </c>
       <c r="B369" s="4" t="n">
-        <v>13758.5</v>
+        <v>16158.5</v>
       </c>
       <c r="C369" s="4" t="n">
-        <v>13243.33429588988</v>
+        <v>15553.47001636346</v>
       </c>
       <c r="D369" t="n">
         <v>1.0389</v>

</xml_diff>